<commit_message>
feat: enhance attendance UI with side panel and status bar, update confidence calculation logic
</commit_message>
<xml_diff>
--- a/Attendance/Attendance.xlsx
+++ b/Attendance/Attendance.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,6 +484,74 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>WIN_20260711_15_13_46_Pro</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>11-07-2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>15:19:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>WIN_20260711_15_14_01_Pro</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>11-07-2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>15:19:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>WIN_20260711_15_14_04_Pro</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>11-07-2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>15:19:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>malay</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>11-07-2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>15:38:53</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: improve face recognition accuracy by augmenting training data and tightening confidence thresholds
</commit_message>
<xml_diff>
--- a/Attendance/Attendance.xlsx
+++ b/Attendance/Attendance.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -552,6 +552,74 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>IMG20260607211840</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>11-07-2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>22:03:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>WIN_20260712_07_33_44_Pro</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>12-07-2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>07:42:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>IMG20260607211840</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>12-07-2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>07:45:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>images (2)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>12-07-2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>07:47:25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: update attendance records and modify emotion detection handling due to import issues
</commit_message>
<xml_diff>
--- a/Attendance/Attendance.xlsx
+++ b/Attendance/Attendance.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -620,6 +620,108 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>images (1)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>12-07-2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>11:57:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>atanu</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>12-07-2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>11:58:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>images</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>12-07-2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>11:58:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>malay</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>12-07-2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>11:58:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>MS_Dhoni_(Prabhav_'23_-_RiGI_2023)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>12-07-2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>11:59:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>12-07-2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>12:12:18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>